<commit_message>
Updated checkout feature files
</commit_message>
<xml_diff>
--- a/DEMOWEBSHOP/src/test/resources/TestData/BillingForm.xlsx
+++ b/DEMOWEBSHOP/src/test/resources/TestData/BillingForm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeeva\OneDrive\Desktop\EXPLEO\Cucumber\AUTOMATIONPROJECT\DEMOWEBSHOP\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F137F4A2-01C8-42DD-BA5D-3A2D6267D21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE6F23F2-55D6-42DC-84F3-90207F1C7ECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1605" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{4DB37D50-0F60-4DFA-9DC0-ADCEFB97BD5E}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="19">
   <si>
     <t>First Name</t>
   </si>
@@ -56,9 +56,6 @@
   </si>
   <si>
     <t>Country</t>
-  </si>
-  <si>
-    <t>state</t>
   </si>
   <si>
     <t>City</t>
@@ -457,13 +454,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{795D27A9-6E91-48D1-B6F1-2C8F583E2011}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="11" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -497,11 +494,8 @@
       <c r="K1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -509,16 +503,16 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2">
-        <v>0</v>
+      <c r="F2" t="s">
+        <v>15</v>
       </c>
       <c r="G2" t="s">
         <v>16</v>
@@ -526,16 +520,13 @@
       <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
-        <v>18</v>
+      <c r="I2">
+        <v>636004</v>
       </c>
       <c r="J2">
-        <v>636004</v>
+        <v>9876543210</v>
       </c>
       <c r="K2">
-        <v>9876543210</v>
-      </c>
-      <c r="L2">
         <v>1234567890</v>
       </c>
     </row>
@@ -549,10 +540,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ADF9D4B-FBF7-4283-A0E8-A560CB59F369}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -586,11 +577,8 @@
       <c r="K1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -598,16 +586,16 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2">
-        <v>0</v>
+      <c r="F2" t="s">
+        <v>15</v>
       </c>
       <c r="G2" t="s">
         <v>16</v>
@@ -615,16 +603,13 @@
       <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
-        <v>18</v>
+      <c r="I2">
+        <v>636004</v>
       </c>
       <c r="J2">
-        <v>636004</v>
+        <v>9876543210</v>
       </c>
       <c r="K2">
-        <v>9876543210</v>
-      </c>
-      <c r="L2">
         <v>1234567890</v>
       </c>
     </row>

</xml_diff>